<commit_message>
Rebuild IG with validation fixes, update ConceptMap canonical URLs
ConceptMap URLs now use http://bw.health.gov/fhir/amr/ConceptMap/
prefix matching the IG canonical. Reduces errors from 122 to 5
(remaining are R4/R4B version mismatches in HL7 dependencies).
Gitignore added for files exceeding GitHub's 100MB limit.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/CodeSystem-botswana-amr-local-method-cs.xlsx
+++ b/output/CodeSystem-botswana-amr-local-method-cs.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://bw.health.gov/fhir/ImplementationGuide/bw-amr-ig/CodeSystem/botswana-amr-local-method-cs</t>
+    <t>http://bw.health.gov/fhir/amr/CodeSystem/botswana-amr-local-method-cs</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T15:05:11-04:00</t>
+    <t>2026-03-13T21:27:21-04:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>